<commit_message>
KFSPTS-38540 update Payment Election template
</commit_message>
<xml_diff>
--- a/src/main/resources/edu/cornell/kfs/cemi/pdp/batch/Payment_Election.xlsx
+++ b/src/main/resources/edu/cornell/kfs/cemi/pdp/batch/Payment_Election.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30524"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nkk4/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://huroncg-my.sharepoint.com/personal/nalder_huronconsultinggroup_com/Documents/Documents/Clover DX/Final Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA0B4E06-F29A-6F45-A2AA-F1805FD028CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA2265E8-3A3A-4713-95F9-857EACDE2A60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35640" yWindow="1140" windowWidth="36400" windowHeight="20460" tabRatio="756" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15390" tabRatio="756" firstSheet="4" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Usage Notes" sheetId="3" state="hidden" r:id="rId1"/>
     <sheet name="Group_ONE" sheetId="2" r:id="rId2"/>
     <sheet name="Group_TWO" sheetId="5" r:id="rId3"/>
-    <sheet name="Group_THREE" sheetId="12" state="hidden" r:id="rId4"/>
-    <sheet name="Group_FOUR" sheetId="13" state="hidden" r:id="rId5"/>
+    <sheet name="Group_THREE" sheetId="12" r:id="rId4"/>
+    <sheet name="Group_FOUR" sheetId="13" r:id="rId5"/>
     <sheet name="Group_ONE_Simple" sheetId="10" state="hidden" r:id="rId6"/>
     <sheet name="Group_THREE_FULL" sheetId="6" state="hidden" r:id="rId7"/>
     <sheet name="Group_FOUR_FULL" sheetId="7" state="hidden" r:id="rId8"/>
@@ -1691,9 +1691,10 @@
         <r>
           <rPr>
             <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
+            <color indexed="8"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
           </rPr>
           <t>Role ID Reference will identify for whom the payment election is created for as well as what role. The ID consists of a type attribute, which should be set to "Employee_ID", "Contingent_Worker_ID", or "Student_ID", and a value attribute, such as "04345”.</t>
         </r>
@@ -6510,7 +6511,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1239" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1199" uniqueCount="307">
   <si>
     <t>Element</t>
   </si>
@@ -7155,289 +7156,286 @@
     <t>Distribution_Balance_1_6</t>
   </si>
   <si>
+    <t>Submit Payment Election Enrollment: Group Two</t>
+  </si>
+  <si>
+    <t>This is the key for this load. Any employee referenced here must also be on the Group One tab.</t>
+  </si>
+  <si>
+    <t>Reference an existing payment election rule, e.g., Payroll, Expense. This rule will apply to all accounts in this group. Recommended to use this tab for Payroll Bonus or another election group that allows multiple elections.</t>
+  </si>
+  <si>
+    <t>default to Expense_Payments</t>
+  </si>
+  <si>
+    <t>leave blank</t>
+  </si>
+  <si>
+    <t>default to TRUE</t>
+  </si>
+  <si>
+    <t>Payment Group Data</t>
+  </si>
+  <si>
+    <t>Payment_Election_Group_Rule_2</t>
+  </si>
+  <si>
+    <t>Payment_Election_Rule_2_1</t>
+  </si>
+  <si>
+    <t>Election_Country_2_1</t>
+  </si>
+  <si>
+    <t>Election_Currency_2_1</t>
+  </si>
+  <si>
+    <t>Payment_Type_2_1</t>
+  </si>
+  <si>
+    <t>Account_Country_2_1</t>
+  </si>
+  <si>
+    <t>Account_Currency_2_1</t>
+  </si>
+  <si>
+    <t>Bank_Account_Nickname_2_1</t>
+  </si>
+  <si>
+    <t>Bank_Account_Name_2_1</t>
+  </si>
+  <si>
+    <t>Account_Number_2_1</t>
+  </si>
+  <si>
+    <t>Account_Type_2_1</t>
+  </si>
+  <si>
+    <t>Bank_Name_2_1</t>
+  </si>
+  <si>
+    <t>Bank_Routing_Number_2_1</t>
+  </si>
+  <si>
+    <t>IBAN_2_1</t>
+  </si>
+  <si>
+    <t>BIC_2_1</t>
+  </si>
+  <si>
+    <t>Branch_Name_2_1</t>
+  </si>
+  <si>
+    <t>Branch_ID_Number_2_1</t>
+  </si>
+  <si>
+    <t>Check_Digit_2_1</t>
+  </si>
+  <si>
+    <t>Distribution_Amount_2_1</t>
+  </si>
+  <si>
+    <t>Distribution_Percentage_2_1</t>
+  </si>
+  <si>
+    <t>Distribution_Balance_2_1</t>
+  </si>
+  <si>
+    <t>Submit Payment Election Enrollment: Group Three</t>
+  </si>
+  <si>
+    <t>Reference an existing payment election rule, e.g., Payroll, Expense. This rule will apply to all accounts in this group. Recommended to use this tab for Expense payments or another election type that allows only one election.</t>
+  </si>
+  <si>
+    <t>Payment_Election_Group_Rule_3</t>
+  </si>
+  <si>
+    <t>Payment_Election_Rule_3</t>
+  </si>
+  <si>
+    <t>Payment_Type_3</t>
+  </si>
+  <si>
+    <t>Account_Number_3</t>
+  </si>
+  <si>
+    <t>Account_Type_3</t>
+  </si>
+  <si>
+    <t>Bank_Name_3</t>
+  </si>
+  <si>
+    <t>Bank_Routing_Number_3</t>
+  </si>
+  <si>
+    <t>Distribution_Amount_3</t>
+  </si>
+  <si>
+    <t>Distribution_Percentage_3</t>
+  </si>
+  <si>
+    <t>Distribution_Balance_3</t>
+  </si>
+  <si>
+    <t>Submit Payment Election Enrollment: Group Four</t>
+  </si>
+  <si>
+    <t>Payment_Election_Group_Rule_4</t>
+  </si>
+  <si>
+    <t>Payment_Election_Rule_4</t>
+  </si>
+  <si>
+    <t>Payment_Type_4</t>
+  </si>
+  <si>
+    <t>Account_Number_4</t>
+  </si>
+  <si>
+    <t>Account_Type_4</t>
+  </si>
+  <si>
+    <t>Bank_Name_4</t>
+  </si>
+  <si>
+    <t>Bank_Routing_Number_4</t>
+  </si>
+  <si>
+    <t>Distribution_Balance_4</t>
+  </si>
+  <si>
+    <t>Review QTR requirements and how that differs from US (IBAN)</t>
+  </si>
+  <si>
     <t>Example Data:</t>
   </si>
   <si>
+    <t>CDXTest-03</t>
+  </si>
+  <si>
+    <t>Regular_Payments</t>
+  </si>
+  <si>
+    <t>DIRECT_DEPOSIT</t>
+  </si>
+  <si>
+    <t>DDA</t>
+  </si>
+  <si>
+    <t>Boston Private Bank</t>
+  </si>
+  <si>
+    <t>011002343</t>
+  </si>
+  <si>
+    <t>SA</t>
+  </si>
+  <si>
+    <t>054001204</t>
+  </si>
+  <si>
+    <t>Must be 1. Defaults to 1 if left blank.</t>
+  </si>
+  <si>
+    <t>Number</t>
+  </si>
+  <si>
+    <t>Order_3</t>
+  </si>
+  <si>
+    <t>Election_Country_3</t>
+  </si>
+  <si>
+    <t>Election_Currency_3</t>
+  </si>
+  <si>
+    <t>Account_Country_3</t>
+  </si>
+  <si>
+    <t>Account_Currency_3</t>
+  </si>
+  <si>
+    <t>Bank_Account_Nickname_3</t>
+  </si>
+  <si>
+    <t>Bank_Account_Name_3</t>
+  </si>
+  <si>
+    <t>IBAN_3</t>
+  </si>
+  <si>
+    <t>BIC_3</t>
+  </si>
+  <si>
+    <t>Branch_Name_3</t>
+  </si>
+  <si>
+    <t>Branch_ID_Number_3</t>
+  </si>
+  <si>
+    <t>Check_Digit_3</t>
+  </si>
+  <si>
     <t>CDXTest-01</t>
   </si>
   <si>
-    <t>DIRECT_DEPOSIT</t>
-  </si>
-  <si>
-    <t>DDA</t>
-  </si>
-  <si>
-    <t>Boston Private Bank</t>
-  </si>
-  <si>
-    <t>011002343</t>
-  </si>
-  <si>
-    <t>SA</t>
-  </si>
-  <si>
-    <t>054001204</t>
-  </si>
-  <si>
-    <t>Submit Payment Election Enrollment: Group Two</t>
-  </si>
-  <si>
-    <t>This is the key for this load. Any employee referenced here must also be on the Group One tab.</t>
-  </si>
-  <si>
-    <t>Reference an existing payment election rule, e.g., Payroll, Expense. This rule will apply to all accounts in this group. Recommended to use this tab for Payroll Bonus or another election group that allows multiple elections.</t>
-  </si>
-  <si>
-    <t>default to Expense_Payments</t>
-  </si>
-  <si>
-    <t>leave blank</t>
-  </si>
-  <si>
-    <t>default to TRUE</t>
-  </si>
-  <si>
-    <t>Payment Group Data</t>
-  </si>
-  <si>
-    <t>Payment_Election_Group_Rule_2</t>
-  </si>
-  <si>
-    <t>Payment_Election_Rule_2_1</t>
-  </si>
-  <si>
-    <t>Election_Country_2_1</t>
-  </si>
-  <si>
-    <t>Election_Currency_2_1</t>
-  </si>
-  <si>
-    <t>Payment_Type_2_1</t>
-  </si>
-  <si>
-    <t>Account_Country_2_1</t>
-  </si>
-  <si>
-    <t>Account_Currency_2_1</t>
-  </si>
-  <si>
-    <t>Bank_Account_Nickname_2_1</t>
-  </si>
-  <si>
-    <t>Bank_Account_Name_2_1</t>
-  </si>
-  <si>
-    <t>Account_Number_2_1</t>
-  </si>
-  <si>
-    <t>Account_Type_2_1</t>
-  </si>
-  <si>
-    <t>Bank_Name_2_1</t>
-  </si>
-  <si>
-    <t>Bank_Routing_Number_2_1</t>
-  </si>
-  <si>
-    <t>IBAN_2_1</t>
-  </si>
-  <si>
-    <t>BIC_2_1</t>
-  </si>
-  <si>
-    <t>Branch_Name_2_1</t>
-  </si>
-  <si>
-    <t>Branch_ID_Number_2_1</t>
-  </si>
-  <si>
-    <t>Check_Digit_2_1</t>
-  </si>
-  <si>
-    <t>Distribution_Amount_2_1</t>
-  </si>
-  <si>
-    <t>Distribution_Percentage_2_1</t>
-  </si>
-  <si>
-    <t>Distribution_Balance_2_1</t>
+    <t>Expense_Payment</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>31256487</t>
+  </si>
+  <si>
+    <t>Citi Bank</t>
   </si>
   <si>
     <t>CDXTest-02</t>
   </si>
   <si>
-    <t>Submit Payment Election Enrollment: Group Three</t>
-  </si>
-  <si>
-    <t>Reference an existing payment election rule, e.g., Payroll, Expense. This rule will apply to all accounts in this group. Recommended to use this tab for Expense payments or another election type that allows only one election.</t>
-  </si>
-  <si>
-    <t>Payment_Election_Group_Rule_3</t>
-  </si>
-  <si>
-    <t>Payment_Election_Rule_3</t>
-  </si>
-  <si>
-    <t>Payment_Type_3</t>
-  </si>
-  <si>
-    <t>Account_Number_3</t>
-  </si>
-  <si>
-    <t>Account_Type_3</t>
-  </si>
-  <si>
-    <t>Bank_Name_3</t>
-  </si>
-  <si>
-    <t>Bank_Routing_Number_3</t>
-  </si>
-  <si>
-    <t>Distribution_Amount_3</t>
-  </si>
-  <si>
-    <t>Distribution_Percentage_3</t>
-  </si>
-  <si>
-    <t>Distribution_Balance_3</t>
-  </si>
-  <si>
-    <t>Expense_Payment</t>
-  </si>
-  <si>
-    <t>31256487</t>
-  </si>
-  <si>
-    <t>Citi Bank</t>
-  </si>
-  <si>
-    <t>CDXTest-03</t>
-  </si>
-  <si>
-    <t>CDXTest-04</t>
-  </si>
-  <si>
-    <t>Submit Payment Election Enrollment: Group Four</t>
-  </si>
-  <si>
-    <t>Payment_Election_Group_Rule_4</t>
-  </si>
-  <si>
-    <t>Payment_Election_Rule_4</t>
-  </si>
-  <si>
-    <t>Payment_Type_4</t>
-  </si>
-  <si>
-    <t>Account_Number_4</t>
-  </si>
-  <si>
-    <t>Account_Type_4</t>
-  </si>
-  <si>
-    <t>Bank_Name_4</t>
-  </si>
-  <si>
-    <t>Bank_Routing_Number_4</t>
-  </si>
-  <si>
-    <t>Distribution_Balance_4</t>
+    <t>Order_4</t>
+  </si>
+  <si>
+    <t>Election_Country_4</t>
+  </si>
+  <si>
+    <t>Election_Currency_4</t>
+  </si>
+  <si>
+    <t>Account_Country_4</t>
+  </si>
+  <si>
+    <t>Account_Currency_4</t>
+  </si>
+  <si>
+    <t>Bank_Account_Nickname_4</t>
+  </si>
+  <si>
+    <t>Bank_Account_Name_4</t>
+  </si>
+  <si>
+    <t>IBAN_4</t>
+  </si>
+  <si>
+    <t>BIC_4</t>
+  </si>
+  <si>
+    <t>Branch_Name_4</t>
+  </si>
+  <si>
+    <t>Branch_ID_Number_4</t>
+  </si>
+  <si>
+    <t>Check_Digit_4</t>
+  </si>
+  <si>
+    <t>Distribution_Amount_4</t>
+  </si>
+  <si>
+    <t>Distribution_Percentage_4</t>
   </si>
   <si>
     <t>Other</t>
-  </si>
-  <si>
-    <t>Review QTR requirements and how that differs from US (IBAN)</t>
-  </si>
-  <si>
-    <t>Regular_Payments</t>
-  </si>
-  <si>
-    <t>Must be 1. Defaults to 1 if left blank.</t>
-  </si>
-  <si>
-    <t>Number</t>
-  </si>
-  <si>
-    <t>Order_3</t>
-  </si>
-  <si>
-    <t>Election_Country_3</t>
-  </si>
-  <si>
-    <t>Election_Currency_3</t>
-  </si>
-  <si>
-    <t>Account_Country_3</t>
-  </si>
-  <si>
-    <t>Account_Currency_3</t>
-  </si>
-  <si>
-    <t>Bank_Account_Nickname_3</t>
-  </si>
-  <si>
-    <t>Bank_Account_Name_3</t>
-  </si>
-  <si>
-    <t>IBAN_3</t>
-  </si>
-  <si>
-    <t>BIC_3</t>
-  </si>
-  <si>
-    <t>Branch_Name_3</t>
-  </si>
-  <si>
-    <t>Branch_ID_Number_3</t>
-  </si>
-  <si>
-    <t>Check_Digit_3</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Order_4</t>
-  </si>
-  <si>
-    <t>Election_Country_4</t>
-  </si>
-  <si>
-    <t>Election_Currency_4</t>
-  </si>
-  <si>
-    <t>Account_Country_4</t>
-  </si>
-  <si>
-    <t>Account_Currency_4</t>
-  </si>
-  <si>
-    <t>Bank_Account_Nickname_4</t>
-  </si>
-  <si>
-    <t>Bank_Account_Name_4</t>
-  </si>
-  <si>
-    <t>IBAN_4</t>
-  </si>
-  <si>
-    <t>BIC_4</t>
-  </si>
-  <si>
-    <t>Branch_Name_4</t>
-  </si>
-  <si>
-    <t>Branch_ID_Number_4</t>
-  </si>
-  <si>
-    <t>Check_Digit_4</t>
-  </si>
-  <si>
-    <t>Distribution_Amount_4</t>
-  </si>
-  <si>
-    <t>Distribution_Percentage_4</t>
   </si>
   <si>
     <t xml:space="preserve">Other </t>
@@ -7453,7 +7451,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -7512,17 +7510,6 @@
       <sz val="6"/>
       <color rgb="FF464646"/>
       <name val="Roboto"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF242424"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -7594,7 +7581,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -7623,10 +7610,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7646,9 +7629,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -7686,7 +7669,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -7792,7 +7775,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -7934,7 +7917,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -7943,14 +7926,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD5E9411-4886-4443-B735-F794B16E117C}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="28.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="97.83203125" customWidth="1"/>
-    <col min="3" max="3" width="106.5" style="1" customWidth="1"/>
+    <col min="1" max="1" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="97.85546875" customWidth="1"/>
+    <col min="3" max="3" width="106.5703125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -7959,7 +7942,7 @@
       </c>
       <c r="C1"/>
     </row>
-    <row r="2" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="57.95">
       <c r="A2" s="8" t="s">
         <v>2</v>
       </c>
@@ -7968,7 +7951,7 @@
       </c>
       <c r="C2"/>
     </row>
-    <row r="3" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="57.95">
       <c r="A3" s="8" t="s">
         <v>4</v>
       </c>
@@ -7977,7 +7960,7 @@
       </c>
       <c r="C3"/>
     </row>
-    <row r="4" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="29.1">
       <c r="A4" s="8" t="s">
         <v>6</v>
       </c>
@@ -7986,7 +7969,7 @@
       </c>
       <c r="C4"/>
     </row>
-    <row r="5" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="29.1">
       <c r="A5" s="8" t="s">
         <v>8</v>
       </c>
@@ -7995,7 +7978,7 @@
       </c>
       <c r="C5"/>
     </row>
-    <row r="6" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3">
       <c r="A6" s="8" t="s">
         <v>10</v>
       </c>
@@ -8004,15 +7987,15 @@
       </c>
       <c r="C6"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3">
       <c r="B7" s="1"/>
       <c r="C7"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3">
       <c r="B8" s="1"/>
       <c r="C8"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3">
       <c r="B9" s="1"/>
       <c r="C9"/>
     </row>
@@ -8023,141 +8006,141 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFB6BE5C-06C9-4E21-B6D2-3A099BD83B31}">
-  <dimension ref="A1:DY7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:DY6"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="24" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.6640625" style="3" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="20.1640625" style="3" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="24.5" style="4" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="18.5" style="4" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="23.5" style="4" customWidth="1"/>
-    <col min="8" max="8" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="27.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.7109375" style="3" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" style="3" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="24.42578125" style="4" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="18.5703125" style="4" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="23.5703125" style="4" customWidth="1"/>
+    <col min="8" max="8" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="35.5" style="4" customWidth="1"/>
-    <col min="17" max="17" width="22.83203125" style="4" customWidth="1"/>
-    <col min="18" max="18" width="21.33203125" style="4" customWidth="1"/>
-    <col min="19" max="19" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="15.33203125" style="4" customWidth="1"/>
-    <col min="23" max="23" width="12.5" style="4" customWidth="1"/>
-    <col min="24" max="24" width="18.33203125" style="4" customWidth="1"/>
-    <col min="25" max="25" width="20.83203125" style="4" customWidth="1"/>
-    <col min="26" max="26" width="18.5" style="4" customWidth="1"/>
-    <col min="27" max="27" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="35.5703125" style="4" customWidth="1"/>
+    <col min="17" max="17" width="22.85546875" style="4" customWidth="1"/>
+    <col min="18" max="18" width="21.28515625" style="4" customWidth="1"/>
+    <col min="19" max="19" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15.28515625" style="4" customWidth="1"/>
+    <col min="23" max="23" width="12.5703125" style="4" customWidth="1"/>
+    <col min="24" max="24" width="18.28515625" style="4" customWidth="1"/>
+    <col min="25" max="25" width="20.85546875" style="4" customWidth="1"/>
+    <col min="26" max="26" width="18.5703125" style="4" customWidth="1"/>
+    <col min="27" max="27" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="22.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="16.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="7.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="6.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="14.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="45" max="45" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="12.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="55" max="55" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="22.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="16.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="7.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="6.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="14.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="65" max="65" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="12.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="75" max="75" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="22.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="16.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="7.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="6.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="14.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="85" max="85" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="12.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="90" max="90" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="92" max="92" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="91" max="91" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="93" max="93" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="94" max="94" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="95" max="95" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="96" max="96" width="22.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="16.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="99" max="99" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="100" max="100" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="101" max="101" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="102" max="102" width="7.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="103" max="103" width="6.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="104" max="104" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="96" max="96" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="97" max="97" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="98" max="98" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="100" max="100" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="102" max="102" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="103" max="103" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="104" max="104" width="14.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="105" max="105" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="106" max="106" width="12.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="107" max="107" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="108" max="108" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="109" max="109" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="110" max="110" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="111" max="111" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="112" max="112" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="113" max="113" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="114" max="114" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="106" max="106" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="107" max="107" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="108" max="108" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="109" max="109" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="110" max="110" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="111" max="111" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="112" max="112" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="113" max="113" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="114" max="114" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="115" max="115" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="116" max="116" width="22.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="117" max="117" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="118" max="118" width="16.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="119" max="119" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="120" max="120" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="121" max="121" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="122" max="122" width="7.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="123" max="123" width="6.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="124" max="124" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="116" max="116" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="117" max="117" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="118" max="118" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="119" max="119" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="120" max="120" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="121" max="121" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="122" max="122" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="123" max="123" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="124" max="124" width="14.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="125" max="125" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="126" max="126" width="12.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="127" max="127" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="128" max="128" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="129" max="129" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="126" max="126" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="127" max="127" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="128" max="128" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="129" max="129" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:129" ht="76" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:129" ht="71.25">
       <c r="A1" s="9" t="s">
         <v>12</v>
       </c>
@@ -8462,7 +8445,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:129" ht="78.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:129" ht="78.75" customHeight="1">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
@@ -8843,7 +8826,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:129" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:129" ht="18">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
@@ -9002,7 +8985,7 @@
       <c r="DX3" s="7"/>
       <c r="DY3" s="7"/>
     </row>
-    <row r="4" spans="1:129" ht="18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:129" ht="18">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -9391,7 +9374,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:129" ht="18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:129" ht="18">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -9780,7 +9763,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:129" ht="18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:129" ht="18">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -10169,118 +10152,8 @@
         <v>209</v>
       </c>
     </row>
-    <row r="7" spans="1:129" x14ac:dyDescent="0.2">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3"/>
-      <c r="P7" s="3"/>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="15"/>
-      <c r="S7" s="3"/>
-      <c r="T7" s="3"/>
-      <c r="U7" s="14"/>
-      <c r="V7" s="3"/>
-      <c r="W7" s="3"/>
-      <c r="X7" s="3"/>
-      <c r="Y7" s="3"/>
-      <c r="Z7" s="3"/>
-      <c r="AD7" s="19"/>
-      <c r="AE7" s="3"/>
-      <c r="AF7" s="3"/>
-      <c r="AG7" s="16"/>
-      <c r="AH7" s="3"/>
-      <c r="AI7" s="3"/>
-      <c r="AJ7" s="3"/>
-      <c r="AK7" s="3"/>
-      <c r="AL7" s="15"/>
-      <c r="AM7" s="3"/>
-      <c r="AN7" s="3"/>
-      <c r="AO7" s="14"/>
-      <c r="AP7" s="3"/>
-      <c r="AQ7" s="3"/>
-      <c r="AR7" s="3"/>
-      <c r="AS7" s="3"/>
-      <c r="AT7" s="3"/>
-      <c r="AX7" s="19"/>
-      <c r="AY7" s="3"/>
-      <c r="AZ7" s="3"/>
-      <c r="BA7" s="16"/>
-      <c r="BB7" s="3"/>
-      <c r="BC7" s="3"/>
-      <c r="BD7" s="3"/>
-      <c r="BE7" s="3"/>
-      <c r="BF7" s="15"/>
-      <c r="BG7" s="3"/>
-      <c r="BH7" s="3"/>
-      <c r="BI7" s="13"/>
-      <c r="BQ7" s="17"/>
-      <c r="BR7" s="19"/>
-      <c r="BS7" s="3"/>
-      <c r="BT7" s="3"/>
-      <c r="BU7" s="16"/>
-      <c r="BV7" s="3"/>
-      <c r="BW7" s="3"/>
-      <c r="BX7" s="3"/>
-      <c r="BY7" s="3"/>
-      <c r="BZ7" s="15"/>
-      <c r="CA7" s="3"/>
-      <c r="CB7" s="3"/>
-      <c r="CC7" s="15"/>
-      <c r="CD7" s="3"/>
-      <c r="CE7" s="3"/>
-      <c r="CF7" s="3"/>
-      <c r="CG7" s="3"/>
-      <c r="CH7" s="3"/>
-      <c r="CK7" s="17"/>
-      <c r="CL7" s="19"/>
-      <c r="CM7" s="3"/>
-      <c r="CN7" s="3"/>
-      <c r="CO7" s="3"/>
-      <c r="CP7" s="3"/>
-      <c r="CQ7" s="3"/>
-      <c r="CR7" s="3"/>
-      <c r="CS7" s="3"/>
-      <c r="CT7" s="15"/>
-      <c r="CU7" s="3"/>
-      <c r="CV7" s="3"/>
-      <c r="CW7" s="15"/>
-      <c r="CX7" s="3"/>
-      <c r="CY7" s="3"/>
-      <c r="CZ7" s="3"/>
-      <c r="DA7" s="3"/>
-      <c r="DB7" s="3"/>
-      <c r="DE7" s="17"/>
-      <c r="DF7" s="19"/>
-      <c r="DG7" s="3"/>
-      <c r="DH7" s="3"/>
-      <c r="DI7" s="3"/>
-      <c r="DJ7" s="3"/>
-      <c r="DK7" s="3"/>
-      <c r="DL7" s="3"/>
-      <c r="DM7" s="3"/>
-      <c r="DN7" s="15"/>
-      <c r="DO7" s="3"/>
-      <c r="DP7" s="3"/>
-      <c r="DQ7" s="15"/>
-      <c r="DR7" s="3"/>
-      <c r="DS7" s="3"/>
-      <c r="DT7" s="3"/>
-      <c r="DU7" s="3"/>
-      <c r="DV7" s="3"/>
-      <c r="DY7" s="17"/>
-    </row>
   </sheetData>
-  <dataValidations count="9">
+  <dataValidations count="7">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="S5 AM5 BG5 CA5 CU5 DO5" xr:uid="{2DBECC3D-94F7-46A8-9FD5-1C3ADF801680}">
       <formula1>"WID,Bank_Account_Type_Code"</formula1>
     </dataValidation>
@@ -10302,12 +10175,6 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F5" xr:uid="{0984F108-43A9-4D62-BD97-52BFC579F006}">
       <formula1>"Contingent_Worker_ID,WID,Employee_ID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="AW7 AC7 DE7 BQ7 CK7 C7:D7 DY7" xr:uid="{46BED44B-5B56-4386-B837-3AF6C08CF1DF}">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AM7 CA7 CU7 BG7 S7 DO7" xr:uid="{1A743E2B-0E3B-4445-87EA-543B37F27A83}">
-      <formula1>"DDA,SA"</formula1>
-    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -10317,43 +10184,43 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C07391C1-ADEA-4783-B088-82B2B03B51C1}">
-  <dimension ref="A1:W10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:W6"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="26.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="73" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:23" ht="71.25">
       <c r="A1" s="9" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>20</v>
@@ -10402,7 +10269,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="65.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:23" ht="65.25" customHeight="1">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
@@ -10410,10 +10277,10 @@
         <v>32</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>36</v>
@@ -10464,21 +10331,21 @@
         <v>47</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="V2" s="5" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:23" ht="18">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="12" t="s">
@@ -10506,7 +10373,7 @@
       <c r="V3" s="7"/>
       <c r="W3" s="7"/>
     </row>
-    <row r="4" spans="1:23" ht="18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:23" ht="18">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -10577,7 +10444,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:23" ht="18">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -10648,7 +10515,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:23" ht="18">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -10656,118 +10523,71 @@
         <v>72</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="K6" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="L6" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="M6" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="N6" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="O6" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="P6" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="Q6" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="R6" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="S6" s="7" t="s">
         <v>233</v>
       </c>
-      <c r="L6" s="7" t="s">
+      <c r="T6" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="M6" s="7" t="s">
+      <c r="U6" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="N6" s="7" t="s">
+      <c r="V6" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="O6" s="7" t="s">
+      <c r="W6" s="7" t="s">
         <v>237</v>
       </c>
-      <c r="P6" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="Q6" s="7" t="s">
-        <v>239</v>
-      </c>
-      <c r="R6" s="7" t="s">
-        <v>240</v>
-      </c>
-      <c r="S6" s="7" t="s">
-        <v>241</v>
-      </c>
-      <c r="T6" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="U6" s="7" t="s">
-        <v>243</v>
-      </c>
-      <c r="V6" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="W6" s="7" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="15"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="14"/>
-      <c r="P7" s="3"/>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="3"/>
-      <c r="S7" s="3"/>
-      <c r="T7" s="3"/>
-    </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="15"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="O8" s="14"/>
-      <c r="P8" s="3"/>
-      <c r="Q8" s="3"/>
-      <c r="R8" s="3"/>
-      <c r="S8" s="3"/>
-      <c r="T8" s="3"/>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A10" s="18"/>
     </row>
   </sheetData>
-  <dataValidations count="8">
+  <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B5" xr:uid="{83B77A8C-5CCD-45B1-933C-EA4E876E5649}">
       <formula1>"Applicant_ID,Contingent_Worker_ID,External_Committee_Member_ID,WID,Candidate_ID,Academic_Person_ID,Student_ID,Employee_ID,Academic_Affiliate_ID,Student_Proxy_ID"</formula1>
     </dataValidation>
@@ -10786,12 +10606,6 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="M5" xr:uid="{2E447897-0F05-4D95-91D9-7FFC2CCBA3AA}">
       <formula1>"WID,Bank_Account_Type_Code"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M7:M8" xr:uid="{6EC7280B-26DA-4C01-A091-A872A667B9E4}">
-      <formula1>"DDA,SA"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="W7:W8" xr:uid="{59C4B4FF-7B57-4E9A-B8B5-230C8DCD6C10}">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -10802,31 +10616,31 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43DC4B2E-DE37-4356-844D-2B6774F3300A}">
   <dimension ref="A1:L9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="26.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.1640625" customWidth="1"/>
-    <col min="11" max="11" width="22.1640625" customWidth="1"/>
-    <col min="12" max="12" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.140625" customWidth="1"/>
+    <col min="11" max="11" width="22.140625" customWidth="1"/>
+    <col min="12" max="12" width="17.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="61" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" ht="64.5">
       <c r="A1" s="9" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>20</v>
@@ -10856,7 +10670,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" ht="18">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
@@ -10872,12 +10686,12 @@
       <c r="K2" s="5"/>
       <c r="L2" s="5"/>
     </row>
-    <row r="3" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" ht="18">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="12"/>
@@ -10890,7 +10704,7 @@
       <c r="K3" s="7"/>
       <c r="L3" s="7"/>
     </row>
-    <row r="4" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="18">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -10928,7 +10742,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" ht="18">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -10966,7 +10780,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" ht="18">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -10974,138 +10788,39 @@
         <v>72</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="L6" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>250</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>251</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>252</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>254</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>255</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>256</v>
-      </c>
-      <c r="K6" s="7" t="s">
-        <v>257</v>
-      </c>
-      <c r="L6" s="7" t="s">
-        <v>258</v>
-      </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>246</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>260</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="I7" s="4">
-        <v>271070801</v>
-      </c>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>260</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="I8" s="4">
-        <v>271070801</v>
-      </c>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>260</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="I9" s="4">
-        <v>271070801</v>
-      </c>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="7" spans="1:12" ht="15"/>
+    <row r="8" spans="1:12" ht="15"/>
+    <row r="9" spans="1:12" ht="15"/>
   </sheetData>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B5" xr:uid="{E4452AC9-BC75-4532-AFD9-7A0592F58770}">
@@ -11129,29 +10844,29 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD03E25A-C84D-4D48-B73D-2E3BC0A89BB0}">
   <dimension ref="A1:J8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="26.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="61" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="54">
       <c r="A1" s="9" t="s">
-        <v>264</v>
+        <v>250</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>20</v>
@@ -11175,7 +10890,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="18">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
@@ -11189,12 +10904,12 @@
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
     </row>
-    <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="18">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="12"/>
@@ -11205,7 +10920,7 @@
       <c r="I3" s="7"/>
       <c r="J3" s="7"/>
     </row>
-    <row r="4" spans="1:10" ht="18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" ht="18">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -11237,7 +10952,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" ht="18">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -11269,7 +10984,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" ht="18">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -11277,102 +10992,34 @@
         <v>72</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>265</v>
+        <v>251</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>266</v>
+        <v>252</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>267</v>
+        <v>253</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>268</v>
+        <v>254</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>269</v>
+        <v>255</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>270</v>
+        <v>256</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>271</v>
+        <v>257</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>272</v>
+        <v>258</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="F7" s="15">
-        <v>987654321</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="I7" s="14" t="s">
-        <v>215</v>
-      </c>
-      <c r="J7" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="F8" s="15">
-        <v>987654321</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="I8" s="14" t="s">
-        <v>215</v>
-      </c>
-      <c r="J8" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="7" spans="1:10" ht="15"/>
+    <row r="8" spans="1:10" ht="15"/>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G7:G8" xr:uid="{C3D63BAB-5790-4BB9-B137-395C6E5B7B5F}">
-      <formula1>"DDA,SA"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J7:J8" xr:uid="{B83AA175-0DD6-4DF1-8509-86B74E2246CB}">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
+  <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G5" xr:uid="{2E77A38B-EBEF-46C8-A1E1-867F045F346D}">
       <formula1>"WID,Bank_Account_Type_Code"</formula1>
     </dataValidation>
@@ -11394,38 +11041,38 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BDF6E9F-389F-4489-BCEB-6DD5879DBE91}">
   <dimension ref="A1:AA7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="24" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.1640625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="16.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.140625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="76" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:27" ht="75">
       <c r="A1" s="9" t="s">
         <v>12</v>
       </c>
@@ -11508,12 +11155,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:27" ht="60" customHeight="1">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>274</v>
+        <v>259</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
@@ -11541,7 +11188,7 @@
       <c r="Z2" s="5"/>
       <c r="AA2" s="5"/>
     </row>
-    <row r="3" spans="1:27" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:27" ht="18">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
@@ -11586,7 +11233,7 @@
       <c r="Z3" s="7"/>
       <c r="AA3" s="7"/>
     </row>
-    <row r="4" spans="1:27" ht="18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:27" ht="18">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -11669,7 +11316,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:27" ht="18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:27" ht="18">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -11752,7 +11399,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:27" ht="18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:27" ht="18">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -11835,66 +11482,66 @@
         <v>149</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:27">
       <c r="A7" s="3" t="s">
-        <v>210</v>
+        <v>260</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>275</v>
-      </c>
       <c r="D7" s="3" t="s">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="E7" s="15">
         <v>987654321</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>213</v>
+        <v>264</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>214</v>
+        <v>265</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>215</v>
+        <v>266</v>
       </c>
       <c r="I7" s="3">
         <v>100</v>
       </c>
       <c r="L7" s="16" t="s">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="M7" s="15">
         <v>1234567890</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>213</v>
+        <v>264</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>214</v>
+        <v>265</v>
       </c>
       <c r="P7" s="14" t="s">
-        <v>215</v>
+        <v>266</v>
       </c>
       <c r="Q7" s="3">
         <v>100</v>
       </c>
       <c r="T7" s="16" t="s">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="U7" s="15">
         <v>123123123</v>
       </c>
       <c r="V7" s="3" t="s">
-        <v>216</v>
+        <v>267</v>
       </c>
       <c r="W7" s="3" t="s">
-        <v>214</v>
+        <v>265</v>
       </c>
       <c r="X7" s="13" t="s">
-        <v>217</v>
+        <v>268</v>
       </c>
       <c r="AA7" s="17" t="b">
         <v>1</v>
@@ -11930,45 +11577,45 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACD0C25A-DB46-45FD-AD1F-9D0E02F210FE}">
   <dimension ref="A1:DD9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="26.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.6640625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="25.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.7109375" style="4" customWidth="1"/>
+    <col min="4" max="4" width="25.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="6.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="19.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="17.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="19.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="17.7109375" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:108" ht="73" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:108" ht="75">
       <c r="A1" s="9" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>20</v>
@@ -12017,7 +11664,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:108" ht="19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:108" ht="18">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
@@ -12045,12 +11692,12 @@
       <c r="W2" s="5"/>
       <c r="X2" s="5"/>
     </row>
-    <row r="3" spans="1:108" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:108" ht="18">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="12" t="s">
@@ -12079,7 +11726,7 @@
       <c r="W3" s="7"/>
       <c r="X3" s="7"/>
     </row>
-    <row r="4" spans="1:108" ht="18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:108" ht="18">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -12153,7 +11800,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:108" ht="18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:108" ht="18">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -12164,7 +11811,7 @@
         <v>77</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="E5" s="8" t="s">
         <v>77</v>
@@ -12227,7 +11874,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:108" ht="18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:108" ht="18">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -12235,101 +11882,101 @@
         <v>72</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="N6" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="P6" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="Q6" s="7" t="s">
+        <v>278</v>
+      </c>
+      <c r="R6" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="S6" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="T6" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="U6" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="V6" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="W6" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="X6" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>278</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>250</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>279</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>280</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>251</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>281</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>282</v>
-      </c>
-      <c r="K6" s="7" t="s">
+    </row>
+    <row r="7" spans="1:108">
+      <c r="A7" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="L6" s="7" t="s">
+      <c r="C7" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="M6" s="7" t="s">
-        <v>252</v>
-      </c>
-      <c r="N6" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="O6" s="7" t="s">
-        <v>254</v>
-      </c>
-      <c r="P6" s="7" t="s">
-        <v>255</v>
-      </c>
-      <c r="Q6" s="7" t="s">
+      <c r="D7" s="4" t="s">
         <v>285</v>
       </c>
-      <c r="R6" s="7" t="s">
-        <v>286</v>
-      </c>
-      <c r="S6" s="7" t="s">
-        <v>287</v>
-      </c>
-      <c r="T6" s="7" t="s">
-        <v>288</v>
-      </c>
-      <c r="U6" s="7" t="s">
-        <v>289</v>
-      </c>
-      <c r="V6" s="7" t="s">
-        <v>256</v>
-      </c>
-      <c r="W6" s="7" t="s">
-        <v>257</v>
-      </c>
-      <c r="X6" s="7" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="7" spans="1:108" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>290</v>
-      </c>
       <c r="E7" s="3" t="s">
-        <v>259</v>
+        <v>284</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3" t="s">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>260</v>
+        <v>286</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>213</v>
+        <v>264</v>
       </c>
       <c r="O7" s="4" t="s">
-        <v>261</v>
+        <v>287</v>
       </c>
       <c r="P7" s="4">
         <v>271070801</v>
@@ -12422,35 +12069,35 @@
       <c r="DC7" s="3"/>
       <c r="DD7" s="3"/>
     </row>
-    <row r="8" spans="1:108" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:108">
       <c r="A8" s="3" t="s">
-        <v>210</v>
+        <v>260</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>246</v>
+        <v>288</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>259</v>
+        <v>284</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>259</v>
+        <v>284</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="H8" s="3" t="s">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>260</v>
+        <v>286</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>213</v>
+        <v>264</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>261</v>
+        <v>287</v>
       </c>
       <c r="P8" s="4">
         <v>271070801</v>
@@ -12543,35 +12190,35 @@
       <c r="DC8" s="3"/>
       <c r="DD8" s="3"/>
     </row>
-    <row r="9" spans="1:108" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:108">
       <c r="A9" s="3" t="s">
-        <v>210</v>
+        <v>260</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>259</v>
+        <v>284</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>259</v>
+        <v>284</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3" t="s">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>260</v>
+        <v>286</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>213</v>
+        <v>264</v>
       </c>
       <c r="O9" s="4" t="s">
-        <v>261</v>
+        <v>287</v>
       </c>
       <c r="P9" s="4">
         <v>271070801</v>
@@ -12694,45 +12341,45 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{589C9B5C-2C65-468C-B018-503470942EE7}">
   <dimension ref="A1:X8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="26.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.6640625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="25.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.7109375" style="4" customWidth="1"/>
+    <col min="4" max="4" width="25.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="6.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="19.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="17.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="19.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="17.7109375" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="73" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" ht="75">
       <c r="A1" s="9" t="s">
-        <v>264</v>
+        <v>250</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>20</v>
@@ -12781,7 +12428,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:24" ht="19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:24" ht="18">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
@@ -12809,12 +12456,12 @@
       <c r="W2" s="5"/>
       <c r="X2" s="5"/>
     </row>
-    <row r="3" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:24" ht="18">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="12" t="s">
@@ -12843,7 +12490,7 @@
       <c r="W3" s="7"/>
       <c r="X3" s="7"/>
     </row>
-    <row r="4" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:24" ht="18">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -12917,7 +12564,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:24" ht="18">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -12928,7 +12575,7 @@
         <v>77</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="E5" s="8" t="s">
         <v>77</v>
@@ -12991,7 +12638,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:24" ht="18">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -12999,112 +12646,112 @@
         <v>72</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>265</v>
+        <v>251</v>
       </c>
       <c r="D6" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="G6" s="7" t="s">
         <v>291</v>
       </c>
-      <c r="E6" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="F6" s="7" t="s">
+      <c r="H6" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="I6" s="7" t="s">
         <v>292</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="J6" s="7" t="s">
         <v>293</v>
       </c>
-      <c r="H6" s="7" t="s">
-        <v>267</v>
-      </c>
-      <c r="I6" s="7" t="s">
+      <c r="K6" s="7" t="s">
         <v>294</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="L6" s="7" t="s">
         <v>295</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="M6" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="N6" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="P6" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="Q6" s="7" t="s">
         <v>296</v>
       </c>
-      <c r="L6" s="7" t="s">
+      <c r="R6" s="7" t="s">
         <v>297</v>
       </c>
-      <c r="M6" s="7" t="s">
-        <v>268</v>
-      </c>
-      <c r="N6" s="7" t="s">
-        <v>269</v>
-      </c>
-      <c r="O6" s="7" t="s">
-        <v>270</v>
-      </c>
-      <c r="P6" s="7" t="s">
-        <v>271</v>
-      </c>
-      <c r="Q6" s="7" t="s">
+      <c r="S6" s="7" t="s">
         <v>298</v>
       </c>
-      <c r="R6" s="7" t="s">
+      <c r="T6" s="7" t="s">
         <v>299</v>
       </c>
-      <c r="S6" s="7" t="s">
+      <c r="U6" s="7" t="s">
         <v>300</v>
       </c>
-      <c r="T6" s="7" t="s">
+      <c r="V6" s="7" t="s">
         <v>301</v>
       </c>
-      <c r="U6" s="7" t="s">
+      <c r="W6" s="7" t="s">
         <v>302</v>
       </c>
-      <c r="V6" s="7" t="s">
+      <c r="X6" s="7" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24">
+      <c r="A7" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>303</v>
-      </c>
-      <c r="W6" s="7" t="s">
-        <v>304</v>
-      </c>
-      <c r="X6" s="7" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>273</v>
       </c>
       <c r="D7" s="3">
         <v>1</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>273</v>
+        <v>303</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3" t="s">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="L7" s="3" t="s">
         <v>305</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>306</v>
       </c>
       <c r="M7" s="15">
         <v>987654321</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>213</v>
+        <v>264</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>214</v>
+        <v>265</v>
       </c>
       <c r="P7" s="14" t="s">
-        <v>215</v>
+        <v>266</v>
       </c>
       <c r="Q7" s="3"/>
       <c r="R7" s="3"/>
@@ -13115,46 +12762,46 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24">
       <c r="A8" s="3" t="s">
-        <v>210</v>
+        <v>260</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>246</v>
+        <v>288</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>273</v>
+        <v>303</v>
       </c>
       <c r="D8" s="3">
         <v>1</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>273</v>
+        <v>303</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="H8" s="3" t="s">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="M8" s="15">
         <v>987654321</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>213</v>
+        <v>264</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>214</v>
+        <v>265</v>
       </c>
       <c r="P8" s="14" t="s">
-        <v>215</v>
+        <v>266</v>
       </c>
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
@@ -13208,8 +12855,8 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B8E5A34B6805674AB42AE8743D903A5B" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f1a81c3d0303786e4db72725a79a1531">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xmlns:ns3="d8c1821b-25b7-4bd3-913e-b4d27807b973" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="399ede5fdaac70f372e865bb1ca16ed3" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B8E5A34B6805674AB42AE8743D903A5B" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="41b35a81783d7de4f664fbd6535a2fc6">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xmlns:ns3="d8c1821b-25b7-4bd3-913e-b4d27807b973" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="157e54fd54b95dd5d963ecaa67584b8e" ns2:_="" ns3:_="">
     <xsd:import namespace="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04"/>
     <xsd:import namespace="d8c1821b-25b7-4bd3-913e-b4d27807b973"/>
     <xsd:element name="properties">
@@ -13236,6 +12883,7 @@
                 <xsd:element ref="ns2:ContentDate" minOccurs="0"/>
                 <xsd:element ref="ns2:Comments" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:Sourceasof" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -13362,6 +13010,11 @@
     <xsd:element name="MediaServiceLocation" ma:index="26" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Sourceasof" ma:index="27" nillable="true" ma:displayName="Source as of" ma:format="DateOnly" ma:internalName="Sourceasof">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -13493,44 +13146,19 @@
     <Comments xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
     <ContentDate xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
     <Status xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04">Draft</Status>
+    <Sourceasof xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6241F7C5-31EE-4E6A-BD4F-9114CB87074C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6241F7C5-31EE-4E6A-BD4F-9114CB87074C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{95BEE76B-B7BD-4FAA-8DC3-5D013A61DA66}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04"/>
-    <ds:schemaRef ds:uri="d8c1821b-25b7-4bd3-913e-b4d27807b973"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BEB67EA2-951B-4ABB-91AE-50DE4DE328E8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2289AEAC-15BB-46FC-8212-B4494D0EED04}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d8c1821b-25b7-4bd3-913e-b4d27807b973"/>
-    <ds:schemaRef ds:uri="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2289AEAC-15BB-46FC-8212-B4494D0EED04}"/>
 </file>
</xml_diff>

<commit_message>
KFSPTS-38540 update Payment Election template (#1978)
</commit_message>
<xml_diff>
--- a/src/main/resources/edu/cornell/kfs/cemi/pdp/batch/Payment_Election.xlsx
+++ b/src/main/resources/edu/cornell/kfs/cemi/pdp/batch/Payment_Election.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30524"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nkk4/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://huroncg-my.sharepoint.com/personal/nalder_huronconsultinggroup_com/Documents/Documents/Clover DX/Final Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA0B4E06-F29A-6F45-A2AA-F1805FD028CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA2265E8-3A3A-4713-95F9-857EACDE2A60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35640" yWindow="1140" windowWidth="36400" windowHeight="20460" tabRatio="756" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15390" tabRatio="756" firstSheet="4" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Usage Notes" sheetId="3" state="hidden" r:id="rId1"/>
     <sheet name="Group_ONE" sheetId="2" r:id="rId2"/>
     <sheet name="Group_TWO" sheetId="5" r:id="rId3"/>
-    <sheet name="Group_THREE" sheetId="12" state="hidden" r:id="rId4"/>
-    <sheet name="Group_FOUR" sheetId="13" state="hidden" r:id="rId5"/>
+    <sheet name="Group_THREE" sheetId="12" r:id="rId4"/>
+    <sheet name="Group_FOUR" sheetId="13" r:id="rId5"/>
     <sheet name="Group_ONE_Simple" sheetId="10" state="hidden" r:id="rId6"/>
     <sheet name="Group_THREE_FULL" sheetId="6" state="hidden" r:id="rId7"/>
     <sheet name="Group_FOUR_FULL" sheetId="7" state="hidden" r:id="rId8"/>
@@ -1691,9 +1691,10 @@
         <r>
           <rPr>
             <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
+            <color indexed="8"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
           </rPr>
           <t>Role ID Reference will identify for whom the payment election is created for as well as what role. The ID consists of a type attribute, which should be set to "Employee_ID", "Contingent_Worker_ID", or "Student_ID", and a value attribute, such as "04345”.</t>
         </r>
@@ -6510,7 +6511,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1239" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1199" uniqueCount="307">
   <si>
     <t>Element</t>
   </si>
@@ -7155,289 +7156,286 @@
     <t>Distribution_Balance_1_6</t>
   </si>
   <si>
+    <t>Submit Payment Election Enrollment: Group Two</t>
+  </si>
+  <si>
+    <t>This is the key for this load. Any employee referenced here must also be on the Group One tab.</t>
+  </si>
+  <si>
+    <t>Reference an existing payment election rule, e.g., Payroll, Expense. This rule will apply to all accounts in this group. Recommended to use this tab for Payroll Bonus or another election group that allows multiple elections.</t>
+  </si>
+  <si>
+    <t>default to Expense_Payments</t>
+  </si>
+  <si>
+    <t>leave blank</t>
+  </si>
+  <si>
+    <t>default to TRUE</t>
+  </si>
+  <si>
+    <t>Payment Group Data</t>
+  </si>
+  <si>
+    <t>Payment_Election_Group_Rule_2</t>
+  </si>
+  <si>
+    <t>Payment_Election_Rule_2_1</t>
+  </si>
+  <si>
+    <t>Election_Country_2_1</t>
+  </si>
+  <si>
+    <t>Election_Currency_2_1</t>
+  </si>
+  <si>
+    <t>Payment_Type_2_1</t>
+  </si>
+  <si>
+    <t>Account_Country_2_1</t>
+  </si>
+  <si>
+    <t>Account_Currency_2_1</t>
+  </si>
+  <si>
+    <t>Bank_Account_Nickname_2_1</t>
+  </si>
+  <si>
+    <t>Bank_Account_Name_2_1</t>
+  </si>
+  <si>
+    <t>Account_Number_2_1</t>
+  </si>
+  <si>
+    <t>Account_Type_2_1</t>
+  </si>
+  <si>
+    <t>Bank_Name_2_1</t>
+  </si>
+  <si>
+    <t>Bank_Routing_Number_2_1</t>
+  </si>
+  <si>
+    <t>IBAN_2_1</t>
+  </si>
+  <si>
+    <t>BIC_2_1</t>
+  </si>
+  <si>
+    <t>Branch_Name_2_1</t>
+  </si>
+  <si>
+    <t>Branch_ID_Number_2_1</t>
+  </si>
+  <si>
+    <t>Check_Digit_2_1</t>
+  </si>
+  <si>
+    <t>Distribution_Amount_2_1</t>
+  </si>
+  <si>
+    <t>Distribution_Percentage_2_1</t>
+  </si>
+  <si>
+    <t>Distribution_Balance_2_1</t>
+  </si>
+  <si>
+    <t>Submit Payment Election Enrollment: Group Three</t>
+  </si>
+  <si>
+    <t>Reference an existing payment election rule, e.g., Payroll, Expense. This rule will apply to all accounts in this group. Recommended to use this tab for Expense payments or another election type that allows only one election.</t>
+  </si>
+  <si>
+    <t>Payment_Election_Group_Rule_3</t>
+  </si>
+  <si>
+    <t>Payment_Election_Rule_3</t>
+  </si>
+  <si>
+    <t>Payment_Type_3</t>
+  </si>
+  <si>
+    <t>Account_Number_3</t>
+  </si>
+  <si>
+    <t>Account_Type_3</t>
+  </si>
+  <si>
+    <t>Bank_Name_3</t>
+  </si>
+  <si>
+    <t>Bank_Routing_Number_3</t>
+  </si>
+  <si>
+    <t>Distribution_Amount_3</t>
+  </si>
+  <si>
+    <t>Distribution_Percentage_3</t>
+  </si>
+  <si>
+    <t>Distribution_Balance_3</t>
+  </si>
+  <si>
+    <t>Submit Payment Election Enrollment: Group Four</t>
+  </si>
+  <si>
+    <t>Payment_Election_Group_Rule_4</t>
+  </si>
+  <si>
+    <t>Payment_Election_Rule_4</t>
+  </si>
+  <si>
+    <t>Payment_Type_4</t>
+  </si>
+  <si>
+    <t>Account_Number_4</t>
+  </si>
+  <si>
+    <t>Account_Type_4</t>
+  </si>
+  <si>
+    <t>Bank_Name_4</t>
+  </si>
+  <si>
+    <t>Bank_Routing_Number_4</t>
+  </si>
+  <si>
+    <t>Distribution_Balance_4</t>
+  </si>
+  <si>
+    <t>Review QTR requirements and how that differs from US (IBAN)</t>
+  </si>
+  <si>
     <t>Example Data:</t>
   </si>
   <si>
+    <t>CDXTest-03</t>
+  </si>
+  <si>
+    <t>Regular_Payments</t>
+  </si>
+  <si>
+    <t>DIRECT_DEPOSIT</t>
+  </si>
+  <si>
+    <t>DDA</t>
+  </si>
+  <si>
+    <t>Boston Private Bank</t>
+  </si>
+  <si>
+    <t>011002343</t>
+  </si>
+  <si>
+    <t>SA</t>
+  </si>
+  <si>
+    <t>054001204</t>
+  </si>
+  <si>
+    <t>Must be 1. Defaults to 1 if left blank.</t>
+  </si>
+  <si>
+    <t>Number</t>
+  </si>
+  <si>
+    <t>Order_3</t>
+  </si>
+  <si>
+    <t>Election_Country_3</t>
+  </si>
+  <si>
+    <t>Election_Currency_3</t>
+  </si>
+  <si>
+    <t>Account_Country_3</t>
+  </si>
+  <si>
+    <t>Account_Currency_3</t>
+  </si>
+  <si>
+    <t>Bank_Account_Nickname_3</t>
+  </si>
+  <si>
+    <t>Bank_Account_Name_3</t>
+  </si>
+  <si>
+    <t>IBAN_3</t>
+  </si>
+  <si>
+    <t>BIC_3</t>
+  </si>
+  <si>
+    <t>Branch_Name_3</t>
+  </si>
+  <si>
+    <t>Branch_ID_Number_3</t>
+  </si>
+  <si>
+    <t>Check_Digit_3</t>
+  </si>
+  <si>
     <t>CDXTest-01</t>
   </si>
   <si>
-    <t>DIRECT_DEPOSIT</t>
-  </si>
-  <si>
-    <t>DDA</t>
-  </si>
-  <si>
-    <t>Boston Private Bank</t>
-  </si>
-  <si>
-    <t>011002343</t>
-  </si>
-  <si>
-    <t>SA</t>
-  </si>
-  <si>
-    <t>054001204</t>
-  </si>
-  <si>
-    <t>Submit Payment Election Enrollment: Group Two</t>
-  </si>
-  <si>
-    <t>This is the key for this load. Any employee referenced here must also be on the Group One tab.</t>
-  </si>
-  <si>
-    <t>Reference an existing payment election rule, e.g., Payroll, Expense. This rule will apply to all accounts in this group. Recommended to use this tab for Payroll Bonus or another election group that allows multiple elections.</t>
-  </si>
-  <si>
-    <t>default to Expense_Payments</t>
-  </si>
-  <si>
-    <t>leave blank</t>
-  </si>
-  <si>
-    <t>default to TRUE</t>
-  </si>
-  <si>
-    <t>Payment Group Data</t>
-  </si>
-  <si>
-    <t>Payment_Election_Group_Rule_2</t>
-  </si>
-  <si>
-    <t>Payment_Election_Rule_2_1</t>
-  </si>
-  <si>
-    <t>Election_Country_2_1</t>
-  </si>
-  <si>
-    <t>Election_Currency_2_1</t>
-  </si>
-  <si>
-    <t>Payment_Type_2_1</t>
-  </si>
-  <si>
-    <t>Account_Country_2_1</t>
-  </si>
-  <si>
-    <t>Account_Currency_2_1</t>
-  </si>
-  <si>
-    <t>Bank_Account_Nickname_2_1</t>
-  </si>
-  <si>
-    <t>Bank_Account_Name_2_1</t>
-  </si>
-  <si>
-    <t>Account_Number_2_1</t>
-  </si>
-  <si>
-    <t>Account_Type_2_1</t>
-  </si>
-  <si>
-    <t>Bank_Name_2_1</t>
-  </si>
-  <si>
-    <t>Bank_Routing_Number_2_1</t>
-  </si>
-  <si>
-    <t>IBAN_2_1</t>
-  </si>
-  <si>
-    <t>BIC_2_1</t>
-  </si>
-  <si>
-    <t>Branch_Name_2_1</t>
-  </si>
-  <si>
-    <t>Branch_ID_Number_2_1</t>
-  </si>
-  <si>
-    <t>Check_Digit_2_1</t>
-  </si>
-  <si>
-    <t>Distribution_Amount_2_1</t>
-  </si>
-  <si>
-    <t>Distribution_Percentage_2_1</t>
-  </si>
-  <si>
-    <t>Distribution_Balance_2_1</t>
+    <t>Expense_Payment</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>31256487</t>
+  </si>
+  <si>
+    <t>Citi Bank</t>
   </si>
   <si>
     <t>CDXTest-02</t>
   </si>
   <si>
-    <t>Submit Payment Election Enrollment: Group Three</t>
-  </si>
-  <si>
-    <t>Reference an existing payment election rule, e.g., Payroll, Expense. This rule will apply to all accounts in this group. Recommended to use this tab for Expense payments or another election type that allows only one election.</t>
-  </si>
-  <si>
-    <t>Payment_Election_Group_Rule_3</t>
-  </si>
-  <si>
-    <t>Payment_Election_Rule_3</t>
-  </si>
-  <si>
-    <t>Payment_Type_3</t>
-  </si>
-  <si>
-    <t>Account_Number_3</t>
-  </si>
-  <si>
-    <t>Account_Type_3</t>
-  </si>
-  <si>
-    <t>Bank_Name_3</t>
-  </si>
-  <si>
-    <t>Bank_Routing_Number_3</t>
-  </si>
-  <si>
-    <t>Distribution_Amount_3</t>
-  </si>
-  <si>
-    <t>Distribution_Percentage_3</t>
-  </si>
-  <si>
-    <t>Distribution_Balance_3</t>
-  </si>
-  <si>
-    <t>Expense_Payment</t>
-  </si>
-  <si>
-    <t>31256487</t>
-  </si>
-  <si>
-    <t>Citi Bank</t>
-  </si>
-  <si>
-    <t>CDXTest-03</t>
-  </si>
-  <si>
-    <t>CDXTest-04</t>
-  </si>
-  <si>
-    <t>Submit Payment Election Enrollment: Group Four</t>
-  </si>
-  <si>
-    <t>Payment_Election_Group_Rule_4</t>
-  </si>
-  <si>
-    <t>Payment_Election_Rule_4</t>
-  </si>
-  <si>
-    <t>Payment_Type_4</t>
-  </si>
-  <si>
-    <t>Account_Number_4</t>
-  </si>
-  <si>
-    <t>Account_Type_4</t>
-  </si>
-  <si>
-    <t>Bank_Name_4</t>
-  </si>
-  <si>
-    <t>Bank_Routing_Number_4</t>
-  </si>
-  <si>
-    <t>Distribution_Balance_4</t>
+    <t>Order_4</t>
+  </si>
+  <si>
+    <t>Election_Country_4</t>
+  </si>
+  <si>
+    <t>Election_Currency_4</t>
+  </si>
+  <si>
+    <t>Account_Country_4</t>
+  </si>
+  <si>
+    <t>Account_Currency_4</t>
+  </si>
+  <si>
+    <t>Bank_Account_Nickname_4</t>
+  </si>
+  <si>
+    <t>Bank_Account_Name_4</t>
+  </si>
+  <si>
+    <t>IBAN_4</t>
+  </si>
+  <si>
+    <t>BIC_4</t>
+  </si>
+  <si>
+    <t>Branch_Name_4</t>
+  </si>
+  <si>
+    <t>Branch_ID_Number_4</t>
+  </si>
+  <si>
+    <t>Check_Digit_4</t>
+  </si>
+  <si>
+    <t>Distribution_Amount_4</t>
+  </si>
+  <si>
+    <t>Distribution_Percentage_4</t>
   </si>
   <si>
     <t>Other</t>
-  </si>
-  <si>
-    <t>Review QTR requirements and how that differs from US (IBAN)</t>
-  </si>
-  <si>
-    <t>Regular_Payments</t>
-  </si>
-  <si>
-    <t>Must be 1. Defaults to 1 if left blank.</t>
-  </si>
-  <si>
-    <t>Number</t>
-  </si>
-  <si>
-    <t>Order_3</t>
-  </si>
-  <si>
-    <t>Election_Country_3</t>
-  </si>
-  <si>
-    <t>Election_Currency_3</t>
-  </si>
-  <si>
-    <t>Account_Country_3</t>
-  </si>
-  <si>
-    <t>Account_Currency_3</t>
-  </si>
-  <si>
-    <t>Bank_Account_Nickname_3</t>
-  </si>
-  <si>
-    <t>Bank_Account_Name_3</t>
-  </si>
-  <si>
-    <t>IBAN_3</t>
-  </si>
-  <si>
-    <t>BIC_3</t>
-  </si>
-  <si>
-    <t>Branch_Name_3</t>
-  </si>
-  <si>
-    <t>Branch_ID_Number_3</t>
-  </si>
-  <si>
-    <t>Check_Digit_3</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Order_4</t>
-  </si>
-  <si>
-    <t>Election_Country_4</t>
-  </si>
-  <si>
-    <t>Election_Currency_4</t>
-  </si>
-  <si>
-    <t>Account_Country_4</t>
-  </si>
-  <si>
-    <t>Account_Currency_4</t>
-  </si>
-  <si>
-    <t>Bank_Account_Nickname_4</t>
-  </si>
-  <si>
-    <t>Bank_Account_Name_4</t>
-  </si>
-  <si>
-    <t>IBAN_4</t>
-  </si>
-  <si>
-    <t>BIC_4</t>
-  </si>
-  <si>
-    <t>Branch_Name_4</t>
-  </si>
-  <si>
-    <t>Branch_ID_Number_4</t>
-  </si>
-  <si>
-    <t>Check_Digit_4</t>
-  </si>
-  <si>
-    <t>Distribution_Amount_4</t>
-  </si>
-  <si>
-    <t>Distribution_Percentage_4</t>
   </si>
   <si>
     <t xml:space="preserve">Other </t>
@@ -7453,7 +7451,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -7512,17 +7510,6 @@
       <sz val="6"/>
       <color rgb="FF464646"/>
       <name val="Roboto"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF242424"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -7594,7 +7581,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -7623,10 +7610,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7646,9 +7629,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -7686,7 +7669,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -7792,7 +7775,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -7934,7 +7917,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -7943,14 +7926,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD5E9411-4886-4443-B735-F794B16E117C}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="28.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="97.83203125" customWidth="1"/>
-    <col min="3" max="3" width="106.5" style="1" customWidth="1"/>
+    <col min="1" max="1" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="97.85546875" customWidth="1"/>
+    <col min="3" max="3" width="106.5703125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -7959,7 +7942,7 @@
       </c>
       <c r="C1"/>
     </row>
-    <row r="2" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="57.95">
       <c r="A2" s="8" t="s">
         <v>2</v>
       </c>
@@ -7968,7 +7951,7 @@
       </c>
       <c r="C2"/>
     </row>
-    <row r="3" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="57.95">
       <c r="A3" s="8" t="s">
         <v>4</v>
       </c>
@@ -7977,7 +7960,7 @@
       </c>
       <c r="C3"/>
     </row>
-    <row r="4" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="29.1">
       <c r="A4" s="8" t="s">
         <v>6</v>
       </c>
@@ -7986,7 +7969,7 @@
       </c>
       <c r="C4"/>
     </row>
-    <row r="5" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="29.1">
       <c r="A5" s="8" t="s">
         <v>8</v>
       </c>
@@ -7995,7 +7978,7 @@
       </c>
       <c r="C5"/>
     </row>
-    <row r="6" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3">
       <c r="A6" s="8" t="s">
         <v>10</v>
       </c>
@@ -8004,15 +7987,15 @@
       </c>
       <c r="C6"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3">
       <c r="B7" s="1"/>
       <c r="C7"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3">
       <c r="B8" s="1"/>
       <c r="C8"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3">
       <c r="B9" s="1"/>
       <c r="C9"/>
     </row>
@@ -8023,141 +8006,141 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFB6BE5C-06C9-4E21-B6D2-3A099BD83B31}">
-  <dimension ref="A1:DY7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:DY6"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="24" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.6640625" style="3" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="20.1640625" style="3" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="24.5" style="4" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="18.5" style="4" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="23.5" style="4" customWidth="1"/>
-    <col min="8" max="8" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="27.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.7109375" style="3" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" style="3" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="24.42578125" style="4" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="18.5703125" style="4" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="23.5703125" style="4" customWidth="1"/>
+    <col min="8" max="8" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="35.5" style="4" customWidth="1"/>
-    <col min="17" max="17" width="22.83203125" style="4" customWidth="1"/>
-    <col min="18" max="18" width="21.33203125" style="4" customWidth="1"/>
-    <col min="19" max="19" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="15.33203125" style="4" customWidth="1"/>
-    <col min="23" max="23" width="12.5" style="4" customWidth="1"/>
-    <col min="24" max="24" width="18.33203125" style="4" customWidth="1"/>
-    <col min="25" max="25" width="20.83203125" style="4" customWidth="1"/>
-    <col min="26" max="26" width="18.5" style="4" customWidth="1"/>
-    <col min="27" max="27" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="35.5703125" style="4" customWidth="1"/>
+    <col min="17" max="17" width="22.85546875" style="4" customWidth="1"/>
+    <col min="18" max="18" width="21.28515625" style="4" customWidth="1"/>
+    <col min="19" max="19" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15.28515625" style="4" customWidth="1"/>
+    <col min="23" max="23" width="12.5703125" style="4" customWidth="1"/>
+    <col min="24" max="24" width="18.28515625" style="4" customWidth="1"/>
+    <col min="25" max="25" width="20.85546875" style="4" customWidth="1"/>
+    <col min="26" max="26" width="18.5703125" style="4" customWidth="1"/>
+    <col min="27" max="27" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="22.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="16.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="7.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="6.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="14.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="45" max="45" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="12.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="55" max="55" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="22.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="16.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="7.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="6.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="14.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="65" max="65" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="12.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="75" max="75" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="22.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="16.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="7.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="6.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="14.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="85" max="85" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="12.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="90" max="90" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="92" max="92" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="91" max="91" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="93" max="93" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="94" max="94" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="95" max="95" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="96" max="96" width="22.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="16.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="99" max="99" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="100" max="100" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="101" max="101" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="102" max="102" width="7.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="103" max="103" width="6.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="104" max="104" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="96" max="96" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="97" max="97" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="98" max="98" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="100" max="100" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="102" max="102" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="103" max="103" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="104" max="104" width="14.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="105" max="105" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="106" max="106" width="12.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="107" max="107" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="108" max="108" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="109" max="109" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="110" max="110" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="111" max="111" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="112" max="112" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="113" max="113" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="114" max="114" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="106" max="106" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="107" max="107" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="108" max="108" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="109" max="109" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="110" max="110" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="111" max="111" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="112" max="112" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="113" max="113" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="114" max="114" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="115" max="115" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="116" max="116" width="22.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="117" max="117" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="118" max="118" width="16.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="119" max="119" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="120" max="120" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="121" max="121" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="122" max="122" width="7.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="123" max="123" width="6.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="124" max="124" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="116" max="116" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="117" max="117" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="118" max="118" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="119" max="119" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="120" max="120" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="121" max="121" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="122" max="122" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="123" max="123" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="124" max="124" width="14.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="125" max="125" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="126" max="126" width="12.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="127" max="127" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="128" max="128" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="129" max="129" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="126" max="126" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="127" max="127" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="128" max="128" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="129" max="129" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:129" ht="76" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:129" ht="71.25">
       <c r="A1" s="9" t="s">
         <v>12</v>
       </c>
@@ -8462,7 +8445,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:129" ht="78.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:129" ht="78.75" customHeight="1">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
@@ -8843,7 +8826,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:129" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:129" ht="18">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
@@ -9002,7 +8985,7 @@
       <c r="DX3" s="7"/>
       <c r="DY3" s="7"/>
     </row>
-    <row r="4" spans="1:129" ht="18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:129" ht="18">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -9391,7 +9374,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:129" ht="18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:129" ht="18">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -9780,7 +9763,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:129" ht="18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:129" ht="18">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -10169,118 +10152,8 @@
         <v>209</v>
       </c>
     </row>
-    <row r="7" spans="1:129" x14ac:dyDescent="0.2">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3"/>
-      <c r="P7" s="3"/>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="15"/>
-      <c r="S7" s="3"/>
-      <c r="T7" s="3"/>
-      <c r="U7" s="14"/>
-      <c r="V7" s="3"/>
-      <c r="W7" s="3"/>
-      <c r="X7" s="3"/>
-      <c r="Y7" s="3"/>
-      <c r="Z7" s="3"/>
-      <c r="AD7" s="19"/>
-      <c r="AE7" s="3"/>
-      <c r="AF7" s="3"/>
-      <c r="AG7" s="16"/>
-      <c r="AH7" s="3"/>
-      <c r="AI7" s="3"/>
-      <c r="AJ7" s="3"/>
-      <c r="AK7" s="3"/>
-      <c r="AL7" s="15"/>
-      <c r="AM7" s="3"/>
-      <c r="AN7" s="3"/>
-      <c r="AO7" s="14"/>
-      <c r="AP7" s="3"/>
-      <c r="AQ7" s="3"/>
-      <c r="AR7" s="3"/>
-      <c r="AS7" s="3"/>
-      <c r="AT7" s="3"/>
-      <c r="AX7" s="19"/>
-      <c r="AY7" s="3"/>
-      <c r="AZ7" s="3"/>
-      <c r="BA7" s="16"/>
-      <c r="BB7" s="3"/>
-      <c r="BC7" s="3"/>
-      <c r="BD7" s="3"/>
-      <c r="BE7" s="3"/>
-      <c r="BF7" s="15"/>
-      <c r="BG7" s="3"/>
-      <c r="BH7" s="3"/>
-      <c r="BI7" s="13"/>
-      <c r="BQ7" s="17"/>
-      <c r="BR7" s="19"/>
-      <c r="BS7" s="3"/>
-      <c r="BT7" s="3"/>
-      <c r="BU7" s="16"/>
-      <c r="BV7" s="3"/>
-      <c r="BW7" s="3"/>
-      <c r="BX7" s="3"/>
-      <c r="BY7" s="3"/>
-      <c r="BZ7" s="15"/>
-      <c r="CA7" s="3"/>
-      <c r="CB7" s="3"/>
-      <c r="CC7" s="15"/>
-      <c r="CD7" s="3"/>
-      <c r="CE7" s="3"/>
-      <c r="CF7" s="3"/>
-      <c r="CG7" s="3"/>
-      <c r="CH7" s="3"/>
-      <c r="CK7" s="17"/>
-      <c r="CL7" s="19"/>
-      <c r="CM7" s="3"/>
-      <c r="CN7" s="3"/>
-      <c r="CO7" s="3"/>
-      <c r="CP7" s="3"/>
-      <c r="CQ7" s="3"/>
-      <c r="CR7" s="3"/>
-      <c r="CS7" s="3"/>
-      <c r="CT7" s="15"/>
-      <c r="CU7" s="3"/>
-      <c r="CV7" s="3"/>
-      <c r="CW7" s="15"/>
-      <c r="CX7" s="3"/>
-      <c r="CY7" s="3"/>
-      <c r="CZ7" s="3"/>
-      <c r="DA7" s="3"/>
-      <c r="DB7" s="3"/>
-      <c r="DE7" s="17"/>
-      <c r="DF7" s="19"/>
-      <c r="DG7" s="3"/>
-      <c r="DH7" s="3"/>
-      <c r="DI7" s="3"/>
-      <c r="DJ7" s="3"/>
-      <c r="DK7" s="3"/>
-      <c r="DL7" s="3"/>
-      <c r="DM7" s="3"/>
-      <c r="DN7" s="15"/>
-      <c r="DO7" s="3"/>
-      <c r="DP7" s="3"/>
-      <c r="DQ7" s="15"/>
-      <c r="DR7" s="3"/>
-      <c r="DS7" s="3"/>
-      <c r="DT7" s="3"/>
-      <c r="DU7" s="3"/>
-      <c r="DV7" s="3"/>
-      <c r="DY7" s="17"/>
-    </row>
   </sheetData>
-  <dataValidations count="9">
+  <dataValidations count="7">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="S5 AM5 BG5 CA5 CU5 DO5" xr:uid="{2DBECC3D-94F7-46A8-9FD5-1C3ADF801680}">
       <formula1>"WID,Bank_Account_Type_Code"</formula1>
     </dataValidation>
@@ -10302,12 +10175,6 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F5" xr:uid="{0984F108-43A9-4D62-BD97-52BFC579F006}">
       <formula1>"Contingent_Worker_ID,WID,Employee_ID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="AW7 AC7 DE7 BQ7 CK7 C7:D7 DY7" xr:uid="{46BED44B-5B56-4386-B837-3AF6C08CF1DF}">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AM7 CA7 CU7 BG7 S7 DO7" xr:uid="{1A743E2B-0E3B-4445-87EA-543B37F27A83}">
-      <formula1>"DDA,SA"</formula1>
-    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -10317,43 +10184,43 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C07391C1-ADEA-4783-B088-82B2B03B51C1}">
-  <dimension ref="A1:W10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:W6"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="26.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="73" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:23" ht="71.25">
       <c r="A1" s="9" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>20</v>
@@ -10402,7 +10269,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="65.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:23" ht="65.25" customHeight="1">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
@@ -10410,10 +10277,10 @@
         <v>32</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>36</v>
@@ -10464,21 +10331,21 @@
         <v>47</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="V2" s="5" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:23" ht="18">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="12" t="s">
@@ -10506,7 +10373,7 @@
       <c r="V3" s="7"/>
       <c r="W3" s="7"/>
     </row>
-    <row r="4" spans="1:23" ht="18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:23" ht="18">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -10577,7 +10444,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:23" ht="18">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -10648,7 +10515,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:23" ht="18">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -10656,118 +10523,71 @@
         <v>72</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="K6" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="L6" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="M6" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="N6" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="O6" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="P6" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="Q6" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="R6" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="S6" s="7" t="s">
         <v>233</v>
       </c>
-      <c r="L6" s="7" t="s">
+      <c r="T6" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="M6" s="7" t="s">
+      <c r="U6" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="N6" s="7" t="s">
+      <c r="V6" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="O6" s="7" t="s">
+      <c r="W6" s="7" t="s">
         <v>237</v>
       </c>
-      <c r="P6" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="Q6" s="7" t="s">
-        <v>239</v>
-      </c>
-      <c r="R6" s="7" t="s">
-        <v>240</v>
-      </c>
-      <c r="S6" s="7" t="s">
-        <v>241</v>
-      </c>
-      <c r="T6" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="U6" s="7" t="s">
-        <v>243</v>
-      </c>
-      <c r="V6" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="W6" s="7" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="15"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="14"/>
-      <c r="P7" s="3"/>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="3"/>
-      <c r="S7" s="3"/>
-      <c r="T7" s="3"/>
-    </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="15"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="O8" s="14"/>
-      <c r="P8" s="3"/>
-      <c r="Q8" s="3"/>
-      <c r="R8" s="3"/>
-      <c r="S8" s="3"/>
-      <c r="T8" s="3"/>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A10" s="18"/>
     </row>
   </sheetData>
-  <dataValidations count="8">
+  <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B5" xr:uid="{83B77A8C-5CCD-45B1-933C-EA4E876E5649}">
       <formula1>"Applicant_ID,Contingent_Worker_ID,External_Committee_Member_ID,WID,Candidate_ID,Academic_Person_ID,Student_ID,Employee_ID,Academic_Affiliate_ID,Student_Proxy_ID"</formula1>
     </dataValidation>
@@ -10786,12 +10606,6 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="M5" xr:uid="{2E447897-0F05-4D95-91D9-7FFC2CCBA3AA}">
       <formula1>"WID,Bank_Account_Type_Code"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M7:M8" xr:uid="{6EC7280B-26DA-4C01-A091-A872A667B9E4}">
-      <formula1>"DDA,SA"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="W7:W8" xr:uid="{59C4B4FF-7B57-4E9A-B8B5-230C8DCD6C10}">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -10802,31 +10616,31 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43DC4B2E-DE37-4356-844D-2B6774F3300A}">
   <dimension ref="A1:L9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="26.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.1640625" customWidth="1"/>
-    <col min="11" max="11" width="22.1640625" customWidth="1"/>
-    <col min="12" max="12" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.140625" customWidth="1"/>
+    <col min="11" max="11" width="22.140625" customWidth="1"/>
+    <col min="12" max="12" width="17.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="61" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" ht="64.5">
       <c r="A1" s="9" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>20</v>
@@ -10856,7 +10670,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" ht="18">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
@@ -10872,12 +10686,12 @@
       <c r="K2" s="5"/>
       <c r="L2" s="5"/>
     </row>
-    <row r="3" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" ht="18">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="12"/>
@@ -10890,7 +10704,7 @@
       <c r="K3" s="7"/>
       <c r="L3" s="7"/>
     </row>
-    <row r="4" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="18">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -10928,7 +10742,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" ht="18">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -10966,7 +10780,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" ht="18">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -10974,138 +10788,39 @@
         <v>72</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="L6" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>250</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>251</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>252</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>254</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>255</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>256</v>
-      </c>
-      <c r="K6" s="7" t="s">
-        <v>257</v>
-      </c>
-      <c r="L6" s="7" t="s">
-        <v>258</v>
-      </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>246</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>260</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="I7" s="4">
-        <v>271070801</v>
-      </c>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>260</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="I8" s="4">
-        <v>271070801</v>
-      </c>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>260</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="I9" s="4">
-        <v>271070801</v>
-      </c>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="7" spans="1:12" ht="15"/>
+    <row r="8" spans="1:12" ht="15"/>
+    <row r="9" spans="1:12" ht="15"/>
   </sheetData>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B5" xr:uid="{E4452AC9-BC75-4532-AFD9-7A0592F58770}">
@@ -11129,29 +10844,29 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD03E25A-C84D-4D48-B73D-2E3BC0A89BB0}">
   <dimension ref="A1:J8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="26.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="61" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="54">
       <c r="A1" s="9" t="s">
-        <v>264</v>
+        <v>250</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>20</v>
@@ -11175,7 +10890,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="18">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
@@ -11189,12 +10904,12 @@
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
     </row>
-    <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="18">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="12"/>
@@ -11205,7 +10920,7 @@
       <c r="I3" s="7"/>
       <c r="J3" s="7"/>
     </row>
-    <row r="4" spans="1:10" ht="18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" ht="18">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -11237,7 +10952,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" ht="18">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -11269,7 +10984,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" ht="18">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -11277,102 +10992,34 @@
         <v>72</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>265</v>
+        <v>251</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>266</v>
+        <v>252</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>267</v>
+        <v>253</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>268</v>
+        <v>254</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>269</v>
+        <v>255</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>270</v>
+        <v>256</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>271</v>
+        <v>257</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>272</v>
+        <v>258</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="F7" s="15">
-        <v>987654321</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="I7" s="14" t="s">
-        <v>215</v>
-      </c>
-      <c r="J7" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="F8" s="15">
-        <v>987654321</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="I8" s="14" t="s">
-        <v>215</v>
-      </c>
-      <c r="J8" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="7" spans="1:10" ht="15"/>
+    <row r="8" spans="1:10" ht="15"/>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G7:G8" xr:uid="{C3D63BAB-5790-4BB9-B137-395C6E5B7B5F}">
-      <formula1>"DDA,SA"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J7:J8" xr:uid="{B83AA175-0DD6-4DF1-8509-86B74E2246CB}">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
+  <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G5" xr:uid="{2E77A38B-EBEF-46C8-A1E1-867F045F346D}">
       <formula1>"WID,Bank_Account_Type_Code"</formula1>
     </dataValidation>
@@ -11394,38 +11041,38 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BDF6E9F-389F-4489-BCEB-6DD5879DBE91}">
   <dimension ref="A1:AA7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="24" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.1640625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="16.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.140625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="76" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:27" ht="75">
       <c r="A1" s="9" t="s">
         <v>12</v>
       </c>
@@ -11508,12 +11155,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:27" ht="60" customHeight="1">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>274</v>
+        <v>259</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
@@ -11541,7 +11188,7 @@
       <c r="Z2" s="5"/>
       <c r="AA2" s="5"/>
     </row>
-    <row r="3" spans="1:27" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:27" ht="18">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
@@ -11586,7 +11233,7 @@
       <c r="Z3" s="7"/>
       <c r="AA3" s="7"/>
     </row>
-    <row r="4" spans="1:27" ht="18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:27" ht="18">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -11669,7 +11316,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:27" ht="18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:27" ht="18">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -11752,7 +11399,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:27" ht="18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:27" ht="18">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -11835,66 +11482,66 @@
         <v>149</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:27">
       <c r="A7" s="3" t="s">
-        <v>210</v>
+        <v>260</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>275</v>
-      </c>
       <c r="D7" s="3" t="s">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="E7" s="15">
         <v>987654321</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>213</v>
+        <v>264</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>214</v>
+        <v>265</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>215</v>
+        <v>266</v>
       </c>
       <c r="I7" s="3">
         <v>100</v>
       </c>
       <c r="L7" s="16" t="s">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="M7" s="15">
         <v>1234567890</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>213</v>
+        <v>264</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>214</v>
+        <v>265</v>
       </c>
       <c r="P7" s="14" t="s">
-        <v>215</v>
+        <v>266</v>
       </c>
       <c r="Q7" s="3">
         <v>100</v>
       </c>
       <c r="T7" s="16" t="s">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="U7" s="15">
         <v>123123123</v>
       </c>
       <c r="V7" s="3" t="s">
-        <v>216</v>
+        <v>267</v>
       </c>
       <c r="W7" s="3" t="s">
-        <v>214</v>
+        <v>265</v>
       </c>
       <c r="X7" s="13" t="s">
-        <v>217</v>
+        <v>268</v>
       </c>
       <c r="AA7" s="17" t="b">
         <v>1</v>
@@ -11930,45 +11577,45 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACD0C25A-DB46-45FD-AD1F-9D0E02F210FE}">
   <dimension ref="A1:DD9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="26.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.6640625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="25.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.7109375" style="4" customWidth="1"/>
+    <col min="4" max="4" width="25.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="6.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="19.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="17.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="19.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="17.7109375" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:108" ht="73" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:108" ht="75">
       <c r="A1" s="9" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>20</v>
@@ -12017,7 +11664,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:108" ht="19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:108" ht="18">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
@@ -12045,12 +11692,12 @@
       <c r="W2" s="5"/>
       <c r="X2" s="5"/>
     </row>
-    <row r="3" spans="1:108" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:108" ht="18">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="12" t="s">
@@ -12079,7 +11726,7 @@
       <c r="W3" s="7"/>
       <c r="X3" s="7"/>
     </row>
-    <row r="4" spans="1:108" ht="18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:108" ht="18">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -12153,7 +11800,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:108" ht="18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:108" ht="18">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -12164,7 +11811,7 @@
         <v>77</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="E5" s="8" t="s">
         <v>77</v>
@@ -12227,7 +11874,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:108" ht="18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:108" ht="18">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -12235,101 +11882,101 @@
         <v>72</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="N6" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="P6" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="Q6" s="7" t="s">
+        <v>278</v>
+      </c>
+      <c r="R6" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="S6" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="T6" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="U6" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="V6" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="W6" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="X6" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>278</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>250</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>279</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>280</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>251</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>281</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>282</v>
-      </c>
-      <c r="K6" s="7" t="s">
+    </row>
+    <row r="7" spans="1:108">
+      <c r="A7" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="L6" s="7" t="s">
+      <c r="C7" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="M6" s="7" t="s">
-        <v>252</v>
-      </c>
-      <c r="N6" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="O6" s="7" t="s">
-        <v>254</v>
-      </c>
-      <c r="P6" s="7" t="s">
-        <v>255</v>
-      </c>
-      <c r="Q6" s="7" t="s">
+      <c r="D7" s="4" t="s">
         <v>285</v>
       </c>
-      <c r="R6" s="7" t="s">
-        <v>286</v>
-      </c>
-      <c r="S6" s="7" t="s">
-        <v>287</v>
-      </c>
-      <c r="T6" s="7" t="s">
-        <v>288</v>
-      </c>
-      <c r="U6" s="7" t="s">
-        <v>289</v>
-      </c>
-      <c r="V6" s="7" t="s">
-        <v>256</v>
-      </c>
-      <c r="W6" s="7" t="s">
-        <v>257</v>
-      </c>
-      <c r="X6" s="7" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="7" spans="1:108" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>290</v>
-      </c>
       <c r="E7" s="3" t="s">
-        <v>259</v>
+        <v>284</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3" t="s">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>260</v>
+        <v>286</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>213</v>
+        <v>264</v>
       </c>
       <c r="O7" s="4" t="s">
-        <v>261</v>
+        <v>287</v>
       </c>
       <c r="P7" s="4">
         <v>271070801</v>
@@ -12422,35 +12069,35 @@
       <c r="DC7" s="3"/>
       <c r="DD7" s="3"/>
     </row>
-    <row r="8" spans="1:108" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:108">
       <c r="A8" s="3" t="s">
-        <v>210</v>
+        <v>260</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>246</v>
+        <v>288</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>259</v>
+        <v>284</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>259</v>
+        <v>284</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="H8" s="3" t="s">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>260</v>
+        <v>286</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>213</v>
+        <v>264</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>261</v>
+        <v>287</v>
       </c>
       <c r="P8" s="4">
         <v>271070801</v>
@@ -12543,35 +12190,35 @@
       <c r="DC8" s="3"/>
       <c r="DD8" s="3"/>
     </row>
-    <row r="9" spans="1:108" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:108">
       <c r="A9" s="3" t="s">
-        <v>210</v>
+        <v>260</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>259</v>
+        <v>284</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>259</v>
+        <v>284</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3" t="s">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>260</v>
+        <v>286</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>213</v>
+        <v>264</v>
       </c>
       <c r="O9" s="4" t="s">
-        <v>261</v>
+        <v>287</v>
       </c>
       <c r="P9" s="4">
         <v>271070801</v>
@@ -12694,45 +12341,45 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{589C9B5C-2C65-468C-B018-503470942EE7}">
   <dimension ref="A1:X8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="26.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.6640625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="25.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.7109375" style="4" customWidth="1"/>
+    <col min="4" max="4" width="25.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="6.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="19.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="17.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="19.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="17.7109375" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="73" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" ht="75">
       <c r="A1" s="9" t="s">
-        <v>264</v>
+        <v>250</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>20</v>
@@ -12781,7 +12428,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:24" ht="19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:24" ht="18">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
@@ -12809,12 +12456,12 @@
       <c r="W2" s="5"/>
       <c r="X2" s="5"/>
     </row>
-    <row r="3" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:24" ht="18">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="12" t="s">
@@ -12843,7 +12490,7 @@
       <c r="W3" s="7"/>
       <c r="X3" s="7"/>
     </row>
-    <row r="4" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:24" ht="18">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -12917,7 +12564,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:24" ht="18">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -12928,7 +12575,7 @@
         <v>77</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="E5" s="8" t="s">
         <v>77</v>
@@ -12991,7 +12638,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:24" ht="18">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -12999,112 +12646,112 @@
         <v>72</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>265</v>
+        <v>251</v>
       </c>
       <c r="D6" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="G6" s="7" t="s">
         <v>291</v>
       </c>
-      <c r="E6" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="F6" s="7" t="s">
+      <c r="H6" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="I6" s="7" t="s">
         <v>292</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="J6" s="7" t="s">
         <v>293</v>
       </c>
-      <c r="H6" s="7" t="s">
-        <v>267</v>
-      </c>
-      <c r="I6" s="7" t="s">
+      <c r="K6" s="7" t="s">
         <v>294</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="L6" s="7" t="s">
         <v>295</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="M6" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="N6" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="P6" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="Q6" s="7" t="s">
         <v>296</v>
       </c>
-      <c r="L6" s="7" t="s">
+      <c r="R6" s="7" t="s">
         <v>297</v>
       </c>
-      <c r="M6" s="7" t="s">
-        <v>268</v>
-      </c>
-      <c r="N6" s="7" t="s">
-        <v>269</v>
-      </c>
-      <c r="O6" s="7" t="s">
-        <v>270</v>
-      </c>
-      <c r="P6" s="7" t="s">
-        <v>271</v>
-      </c>
-      <c r="Q6" s="7" t="s">
+      <c r="S6" s="7" t="s">
         <v>298</v>
       </c>
-      <c r="R6" s="7" t="s">
+      <c r="T6" s="7" t="s">
         <v>299</v>
       </c>
-      <c r="S6" s="7" t="s">
+      <c r="U6" s="7" t="s">
         <v>300</v>
       </c>
-      <c r="T6" s="7" t="s">
+      <c r="V6" s="7" t="s">
         <v>301</v>
       </c>
-      <c r="U6" s="7" t="s">
+      <c r="W6" s="7" t="s">
         <v>302</v>
       </c>
-      <c r="V6" s="7" t="s">
+      <c r="X6" s="7" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24">
+      <c r="A7" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>303</v>
-      </c>
-      <c r="W6" s="7" t="s">
-        <v>304</v>
-      </c>
-      <c r="X6" s="7" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>273</v>
       </c>
       <c r="D7" s="3">
         <v>1</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>273</v>
+        <v>303</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3" t="s">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="L7" s="3" t="s">
         <v>305</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>306</v>
       </c>
       <c r="M7" s="15">
         <v>987654321</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>213</v>
+        <v>264</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>214</v>
+        <v>265</v>
       </c>
       <c r="P7" s="14" t="s">
-        <v>215</v>
+        <v>266</v>
       </c>
       <c r="Q7" s="3"/>
       <c r="R7" s="3"/>
@@ -13115,46 +12762,46 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24">
       <c r="A8" s="3" t="s">
-        <v>210</v>
+        <v>260</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>246</v>
+        <v>288</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>273</v>
+        <v>303</v>
       </c>
       <c r="D8" s="3">
         <v>1</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>273</v>
+        <v>303</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="H8" s="3" t="s">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="M8" s="15">
         <v>987654321</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>213</v>
+        <v>264</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>214</v>
+        <v>265</v>
       </c>
       <c r="P8" s="14" t="s">
-        <v>215</v>
+        <v>266</v>
       </c>
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
@@ -13208,8 +12855,8 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B8E5A34B6805674AB42AE8743D903A5B" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f1a81c3d0303786e4db72725a79a1531">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xmlns:ns3="d8c1821b-25b7-4bd3-913e-b4d27807b973" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="399ede5fdaac70f372e865bb1ca16ed3" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B8E5A34B6805674AB42AE8743D903A5B" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="41b35a81783d7de4f664fbd6535a2fc6">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xmlns:ns3="d8c1821b-25b7-4bd3-913e-b4d27807b973" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="157e54fd54b95dd5d963ecaa67584b8e" ns2:_="" ns3:_="">
     <xsd:import namespace="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04"/>
     <xsd:import namespace="d8c1821b-25b7-4bd3-913e-b4d27807b973"/>
     <xsd:element name="properties">
@@ -13236,6 +12883,7 @@
                 <xsd:element ref="ns2:ContentDate" minOccurs="0"/>
                 <xsd:element ref="ns2:Comments" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:Sourceasof" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -13362,6 +13010,11 @@
     <xsd:element name="MediaServiceLocation" ma:index="26" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Sourceasof" ma:index="27" nillable="true" ma:displayName="Source as of" ma:format="DateOnly" ma:internalName="Sourceasof">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -13493,44 +13146,19 @@
     <Comments xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
     <ContentDate xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
     <Status xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04">Draft</Status>
+    <Sourceasof xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6241F7C5-31EE-4E6A-BD4F-9114CB87074C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6241F7C5-31EE-4E6A-BD4F-9114CB87074C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{95BEE76B-B7BD-4FAA-8DC3-5D013A61DA66}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04"/>
-    <ds:schemaRef ds:uri="d8c1821b-25b7-4bd3-913e-b4d27807b973"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BEB67EA2-951B-4ABB-91AE-50DE4DE328E8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2289AEAC-15BB-46FC-8212-B4494D0EED04}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d8c1821b-25b7-4bd3-913e-b4d27807b973"/>
-    <ds:schemaRef ds:uri="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2289AEAC-15BB-46FC-8212-B4494D0EED04}"/>
 </file>
</xml_diff>